<commit_message>
fix: align bulk import parameter columns
Places each K1-K7 parameter code before its Chinese and English descriptions, preserves bilingual option data, and skips template examples during imports.
</commit_message>
<xml_diff>
--- a/cloud/public/产品导入标准表格.xlsx
+++ b/cloud/public/产品导入标准表格.xlsx
@@ -559,107 +559,107 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>参数1编码</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>参数1名称(中)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>参数1名称(英)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>参数1编码</t>
-        </is>
-      </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>参数2编码</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>参数2名称(中)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>参数2名称(英)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>参数2编码</t>
-        </is>
-      </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>参数3编码</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>参数3名称(中)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>参数3名称(英)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>参数3编码</t>
-        </is>
-      </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>参数4编码</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>参数4名称(中)</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>参数4名称(英)</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>参数4编码</t>
-        </is>
-      </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
+          <t>参数5编码</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>参数5名称(中)</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>参数5名称(英)</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>参数5编码</t>
-        </is>
-      </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
+          <t>参数6编码</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
           <t>参数6名称(中)</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>参数6名称(英)</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>参数6编码</t>
-        </is>
-      </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
+          <t>参数7编码</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
           <t>参数7名称(中)</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>参数7名称(英)</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>参数7编码</t>
         </is>
       </c>
     </row>
@@ -696,62 +696,62 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
           <t>不锈钢</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Staines Steel</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
           <t>A24090</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>A24090</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
           <t>AISI 316不锈钢</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>AISI 316 Stainless Steel</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
           <t>生产工艺：铸造-加工-抛丸-酸洗-电解抛光-钝化-封闭</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>Production process: Casting - processing - shot blasting - pickling - electrolytic polishing - passivation - sealing</t>
-        </is>
-      </c>
-      <c r="R2" s="2" t="inlineStr">
-        <is>
-          <t>04</t>
         </is>
       </c>
     </row>
@@ -788,17 +788,17 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
           <t>碳钢</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Carbon Steel</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>05</t>
         </is>
       </c>
     </row>
@@ -835,32 +835,32 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
           <t>外径</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>OD</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
-      </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
+          <t>J5</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
           <t>钢级</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Grade</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>J5</t>
         </is>
       </c>
     </row>
@@ -897,15 +897,17 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>磅级</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-    </row>
+      <c r="I5" s="2" t="n"/>
+    </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
@@ -956,7 +958,7 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">   参数1~7：每个参数 3 列 = 名称(中) + 名称(英) + 编码</t>
+          <t xml:space="preserve">   参数1~7：每个参数 3 列 = 编码 + 名称(中) + 名称(英)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: preserve import translations
Separates parameter group names from option values for 41-column imports while retaining 27-column compatibility. Repairs legacy group translations when bilingual values were duplicated.
</commit_message>
<xml_diff>
--- a/cloud/public/产品导入标准表格.xlsx
+++ b/cloud/public/产品导入标准表格.xlsx
@@ -10,7 +10,9 @@
     <sheet name="产品导入" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="填写说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'产品导入'!$A$1:$AO$2</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -18,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,8 +64,12 @@
       <color rgb="00111827"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -78,6 +84,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0017365D"/>
       </patternFill>
     </fill>
   </fills>
@@ -107,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -127,6 +138,19 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -494,428 +518,613 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA7"/>
+  <dimension ref="A1:AO300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="14" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
-    <col width="14" customWidth="1" min="24" max="24"/>
-    <col width="14" customWidth="1" min="25" max="25"/>
-    <col width="14" customWidth="1" min="26" max="26"/>
-    <col width="14" customWidth="1" min="27" max="27"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="25" max="25"/>
+    <col width="18" customWidth="1" min="26" max="26"/>
+    <col width="18" customWidth="1" min="27" max="27"/>
+    <col width="18" customWidth="1" min="28" max="28"/>
+    <col width="18" customWidth="1" min="29" max="29"/>
+    <col width="18" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="18" customWidth="1" min="32" max="32"/>
+    <col width="18" customWidth="1" min="33" max="33"/>
+    <col width="18" customWidth="1" min="34" max="34"/>
+    <col width="18" customWidth="1" min="35" max="35"/>
+    <col width="18" customWidth="1" min="36" max="36"/>
+    <col width="18" customWidth="1" min="37" max="37"/>
+    <col width="18" customWidth="1" min="38" max="38"/>
+    <col width="18" customWidth="1" min="39" max="39"/>
+    <col width="18" customWidth="1" min="40" max="40"/>
+    <col width="18" customWidth="1" min="41" max="41"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>产品标准(中)</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>产品标准(英)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>产品分类(中)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>产品分类(英)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>产品名称(中)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>产品名称(英)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>参数1分类名称(中)</t>
+        </is>
+      </c>
+      <c r="H1" s="11" t="inlineStr">
+        <is>
+          <t>参数1分类名称(英)</t>
+        </is>
+      </c>
+      <c r="I1" s="11" t="inlineStr">
         <is>
           <t>参数1编码</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="11" t="inlineStr">
         <is>
           <t>参数1名称(中)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="11" t="inlineStr">
         <is>
           <t>参数1名称(英)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="11" t="inlineStr">
+        <is>
+          <t>参数2分类名称(中)</t>
+        </is>
+      </c>
+      <c r="M1" s="11" t="inlineStr">
+        <is>
+          <t>参数2分类名称(英)</t>
+        </is>
+      </c>
+      <c r="N1" s="11" t="inlineStr">
         <is>
           <t>参数2编码</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="O1" s="11" t="inlineStr">
         <is>
           <t>参数2名称(中)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="P1" s="11" t="inlineStr">
         <is>
           <t>参数2名称(英)</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="Q1" s="11" t="inlineStr">
+        <is>
+          <t>参数3分类名称(中)</t>
+        </is>
+      </c>
+      <c r="R1" s="11" t="inlineStr">
+        <is>
+          <t>参数3分类名称(英)</t>
+        </is>
+      </c>
+      <c r="S1" s="11" t="inlineStr">
         <is>
           <t>参数3编码</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="T1" s="11" t="inlineStr">
         <is>
           <t>参数3名称(中)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="U1" s="11" t="inlineStr">
         <is>
           <t>参数3名称(英)</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="V1" s="11" t="inlineStr">
+        <is>
+          <t>参数4分类名称(中)</t>
+        </is>
+      </c>
+      <c r="W1" s="11" t="inlineStr">
+        <is>
+          <t>参数4分类名称(英)</t>
+        </is>
+      </c>
+      <c r="X1" s="11" t="inlineStr">
         <is>
           <t>参数4编码</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Y1" s="11" t="inlineStr">
         <is>
           <t>参数4名称(中)</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="Z1" s="11" t="inlineStr">
         <is>
           <t>参数4名称(英)</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="AA1" s="11" t="inlineStr">
+        <is>
+          <t>参数5分类名称(中)</t>
+        </is>
+      </c>
+      <c r="AB1" s="12" t="inlineStr">
+        <is>
+          <t>参数5分类名称(英)</t>
+        </is>
+      </c>
+      <c r="AC1" s="12" t="inlineStr">
         <is>
           <t>参数5编码</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="AD1" s="12" t="inlineStr">
         <is>
           <t>参数5名称(中)</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="AE1" s="12" t="inlineStr">
         <is>
           <t>参数5名称(英)</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AF1" s="12" t="inlineStr">
+        <is>
+          <t>参数6分类名称(中)</t>
+        </is>
+      </c>
+      <c r="AG1" s="12" t="inlineStr">
+        <is>
+          <t>参数6分类名称(英)</t>
+        </is>
+      </c>
+      <c r="AH1" s="12" t="inlineStr">
         <is>
           <t>参数6编码</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AI1" s="12" t="inlineStr">
         <is>
           <t>参数6名称(中)</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AJ1" s="12" t="inlineStr">
         <is>
           <t>参数6名称(英)</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AK1" s="12" t="inlineStr">
+        <is>
+          <t>参数7分类名称(中)</t>
+        </is>
+      </c>
+      <c r="AL1" s="12" t="inlineStr">
+        <is>
+          <t>参数7分类名称(英)</t>
+        </is>
+      </c>
+      <c r="AM1" s="12" t="inlineStr">
         <is>
           <t>参数7编码</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AN1" s="12" t="inlineStr">
         <is>
           <t>参数7名称(中)</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AO1" s="12" t="inlineStr">
         <is>
           <t>参数7名称(英)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>机械</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Mechanical Products</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>铸造</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Casting</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>精铸</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Precision Casting</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>不锈钢</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Staines Steel</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>A24090</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>A24090</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>AISI 316不锈钢</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>AISI 316 Stainless Steel</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="inlineStr">
-        <is>
-          <t>生产工艺：铸造-加工-抛丸-酸洗-电解抛光-钝化-封闭</t>
-        </is>
-      </c>
-      <c r="R2" s="2" t="inlineStr">
-        <is>
-          <t>Production process: Casting - processing - shot blasting - pickling - electrolytic polishing - passivation - sealing</t>
-        </is>
-      </c>
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>机械</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Mechanical Products</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>铸造</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Casting</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>精铸</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Precision Casting</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>碳钢</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Carbon Steel</t>
-        </is>
-      </c>
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>套管和油管</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>API 5CT</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>套管</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Casing</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>套管</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Casing</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>外径</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>OD</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>J5</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>钢级</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>Grade</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="n"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" s="2" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>套管和油管</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>API 5CT</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>油管</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Tubing</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>油管</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Tubing</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>磅级</t>
-        </is>
-      </c>
+      <c r="A5" s="2" t="n"/>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
       <c r="I5" s="2" t="n"/>
     </row>
     <row r="6"/>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>以上黄色行为示例，请删除后填写真实数据</t>
-        </is>
-      </c>
+      <c r="A7" s="7" t="n"/>
     </row>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
+    <row r="214"/>
+    <row r="215"/>
+    <row r="216"/>
+    <row r="217"/>
+    <row r="218"/>
+    <row r="219"/>
+    <row r="220"/>
+    <row r="221"/>
+    <row r="222"/>
+    <row r="223"/>
+    <row r="224"/>
+    <row r="225"/>
+    <row r="226"/>
+    <row r="227"/>
+    <row r="228"/>
+    <row r="229"/>
+    <row r="230"/>
+    <row r="231"/>
+    <row r="232"/>
+    <row r="233"/>
+    <row r="234"/>
+    <row r="235"/>
+    <row r="236"/>
+    <row r="237"/>
+    <row r="238"/>
+    <row r="239"/>
+    <row r="240"/>
+    <row r="241"/>
+    <row r="242"/>
+    <row r="243"/>
+    <row r="244"/>
+    <row r="245"/>
+    <row r="246"/>
+    <row r="247"/>
+    <row r="248"/>
+    <row r="249"/>
+    <row r="250"/>
+    <row r="251"/>
+    <row r="252"/>
+    <row r="253"/>
+    <row r="254"/>
+    <row r="255"/>
+    <row r="256"/>
+    <row r="257"/>
+    <row r="258"/>
+    <row r="259"/>
+    <row r="260"/>
+    <row r="261"/>
+    <row r="262"/>
+    <row r="263"/>
+    <row r="264"/>
+    <row r="265"/>
+    <row r="266"/>
+    <row r="267"/>
+    <row r="268"/>
+    <row r="269"/>
+    <row r="270"/>
+    <row r="271"/>
+    <row r="272"/>
+    <row r="273"/>
+    <row r="274"/>
+    <row r="275"/>
+    <row r="276"/>
+    <row r="277"/>
+    <row r="278"/>
+    <row r="279"/>
+    <row r="280"/>
+    <row r="281"/>
+    <row r="282"/>
+    <row r="283"/>
+    <row r="284"/>
+    <row r="285"/>
+    <row r="286"/>
+    <row r="287"/>
+    <row r="288"/>
+    <row r="289"/>
+    <row r="290"/>
+    <row r="291"/>
+    <row r="292"/>
+    <row r="293"/>
+    <row r="294"/>
+    <row r="295"/>
+    <row r="296"/>
+    <row r="297"/>
+    <row r="298"/>
+    <row r="299"/>
+    <row r="300"/>
   </sheetData>
+  <autoFilter ref="A1:AO2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -926,130 +1135,90 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="120" customWidth="1" min="1" max="1"/>
-    <col width="118" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="112" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="8" t="inlineStr">
-        <is>
-          <t>Vigor 编码器 - 产品批量导入填写说明</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr"/>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Vigor 产品编码器 - 批量导入填写说明</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr"/>
     </row>
-    <row r="2">
-      <c r="A2" s="9" t="inlineStr">
-        <is>
-          <t>一、表格结构：一行 = 一个产品</t>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1. 产品层级</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>填写产品标准、产品分类、产品名称的中英文。系统自动分配标准、分类和产品编码。</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   A~F 列：产品标准(中/英)、产品分类(中/英)、产品名称(中/英) —— 产品归属的层级</t>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2. K1-K7 结构</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>每组固定为：参数分类名称(中) → 参数分类名称(英) → 参数编码 → 参数名称(中) → 参数名称(英)。</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   参数1~7：每个参数 3 列 = 编码 + 名称(中) + 名称(英)</t>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3. 参数分类名称</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>填写参数类别，如“外径 / O.D.”、“钢级 / Grade”、“长度 / Length”、“螺纹类型 / Thread”。同一产品、同一 K 组应保持一致。</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       名称(中/英)：该参数值的中英文描述（如 不锈钢 / Staines Steel），可只填一个</t>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4. 参数选项</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>“参数编码”对应一个选项的自定义编码；“参数名称(中/英)”对应该编码的具体参数值。使用多行可录入同一 K 组的多个选项。</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       编码：参数值的自定义编码（如 01），会拼进完整产品编码，同参数内不可重复</t>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5. 英文原则</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>产品层级、参数分类、参数选项的中英文独立保存。没有经过确认的英文请留空。</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>二、Sheet1 黄色示例行说明</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   行2 精铸：4 个参数完整填写（材料/牌号/材质/工艺，编码 01~04）-&gt; 编码 PAAA01020304</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   行3 精铸（同行2 产品）：参数1 再填 碳钢/05 -&gt; 参数1 有 2 个可选值：01 不锈钢、05 碳钢</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   行4 套管：只填 2 个参数（外径 45、钢级 J5），其余留空</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   行5 油管：只填中文（磅级/12），英文留空</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>三、填写规则</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   编码自动生成：标准/分类 A~Z、产品 AA~ZZ，无需填写</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   重复导入：按中文名匹配复用，只补充新选项，不重复创建</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   多选项：同一产品同一参数列，多行填不同值即增加可选值</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>四、操作步骤</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   1) 删除黄色示例行 2) 填写数据 3) 数据管理页顶部「批量导入」选此文件 4) 自动导入完成</t>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>6. 空参数组</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>未使用的 K5-K7 整组保持空白。</t>
         </is>
       </c>
     </row>

</xml_diff>